<commit_message>
Update example test file RegularAutoFilter
Update reference test file for example RegularAutoFilter. After style
infrastructure switch, the styles part is saved differently.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/AutoFilter/RegularAutoFilter.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/AutoFilter/RegularAutoFilter.xlsx
@@ -79,61 +79,53 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -818,7 +810,7 @@
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="0">
+      <x:c r="A8" s="1">
         <x:f>SUBTOTAL(109,[Numbers])</x:f>
       </x:c>
     </x:row>

</xml_diff>